<commit_message>
Add dashboard functionality and cleanup old Claude agents
- Created new Streamlit dashboard for FBA analysis
- Removed deprecated .claude/agents_0 and commands_0 directories
- Updated project configuration and documentation
- Added comprehensive analysis reports and memories
- Integrated Amazon FBA profit calculation tools
- Enhanced state management and browser automation

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/YT -  Amazon FBA Profit Calculatort vat reg.xlsx
+++ b/YT -  Amazon FBA Profit Calculatort vat reg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Desktop\Amazon-FBA-Agent-System-v32 - latest good - Copy (8) - Copy - Copy - POSTLONGRUNPREKIRO2 beforecompletion-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{24D2B647-DBD7-4930-B3C0-CF0B920F49C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A45C632-EE29-482F-904E-55507CD70638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -126,30 +126,35 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="5"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="4"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -548,8 +553,7 @@
         <v>15</v>
       </c>
       <c r="B3" s="4">
-        <f>1.36*1.2</f>
-        <v>1.6320000000000001</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -557,7 +561,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="4">
-        <v>6</v>
+        <v>10.73</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -565,7 +569,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="4">
-        <v>2.85</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -573,7 +577,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="4">
-        <v>0.78</v>
+        <v>3.04</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -581,7 +585,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="4">
-        <v>0.55000000000000004</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -606,7 +610,7 @@
       </c>
       <c r="B11" s="9">
         <f>B4*20/120</f>
-        <v>1</v>
+        <v>1.7883333333333336</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -615,7 +619,7 @@
       </c>
       <c r="B12" s="9">
         <f>(B3/1.2)*20%</f>
-        <v>0.27200000000000002</v>
+        <v>0.3833333333333333</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -624,7 +628,7 @@
       </c>
       <c r="B13" s="10">
         <f>B4-B5-B6-B11</f>
-        <v>1.37</v>
+        <v>4.2916666666666679</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -633,7 +637,7 @@
       </c>
       <c r="B14" s="10">
         <f>B11-B12</f>
-        <v>0.72799999999999998</v>
+        <v>1.4050000000000002</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -642,7 +646,7 @@
       </c>
       <c r="B15" s="11">
         <f>(B13-(B3/1.2)-B7-B8)</f>
-        <v>-0.54</v>
+        <v>1.7750000000000012</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -650,8 +654,8 @@
         <v>12</v>
       </c>
       <c r="B16" s="12">
-        <f>B15/(B3/1.2)</f>
-        <v>-0.39705882352941174</v>
+        <f>B15/((B3/1.2)+B7)</f>
+        <v>0.70529801324503361</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
@@ -660,7 +664,7 @@
       </c>
       <c r="B17" s="13">
         <f>(B4-B11-B15)</f>
-        <v>5.54</v>
+        <v>7.1666666666666652</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
@@ -669,7 +673,7 @@
       </c>
       <c r="B18" s="12">
         <f>(B15/(B4/1.2))</f>
-        <v>-0.10800000000000001</v>
+        <v>0.19850885368126758</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
@@ -741,7 +745,7 @@
       </c>
       <c r="B34" s="23">
         <f>((B16))</f>
-        <v>-0.39705882352941174</v>
+        <v>0.70529801324503361</v>
       </c>
       <c r="C34" s="19"/>
       <c r="D34" s="19"/>
@@ -752,7 +756,7 @@
       </c>
       <c r="B35" s="23">
         <f t="shared" ref="B35:B38" si="0">B18*20%</f>
-        <v>-2.1600000000000005E-2</v>
+        <v>3.9701770736253521E-2</v>
       </c>
       <c r="C35" s="19"/>
       <c r="D35" s="19"/>
@@ -794,7 +798,7 @@
       </c>
       <c r="B39" s="25">
         <f>(B17-(B18+B19+B20+B21+B35+B36+B37+B38))</f>
-        <v>5.6696</v>
+        <v>6.9284560422491444</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -803,7 +807,7 @@
       </c>
       <c r="B40" s="26">
         <f>(B39-(B16))</f>
-        <v>6.0666588235294121</v>
+        <v>6.2231580290041109</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -812,7 +816,7 @@
       </c>
       <c r="B41" s="27">
         <f>B40/(B16)</f>
-        <v>-15.278992592592594</v>
+        <v>8.823444717179532</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -821,7 +825,7 @@
       </c>
       <c r="B42" s="28">
         <f>B17-B40</f>
-        <v>-0.52665882352941207</v>
+        <v>0.94350863766255433</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -830,7 +834,7 @@
       </c>
       <c r="B43" s="30">
         <f>B40/B17</f>
-        <v>1.0950647695901465</v>
+        <v>0.86834763195406217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>